<commit_message>
changement et correction des different filtre pour l'affichage des fiches des postes
</commit_message>
<xml_diff>
--- a/fiches_de_poste.xlsx
+++ b/fiches_de_poste.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-03-21</t>
+          <t>21/03/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Piste identifiée</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>20/03/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2025-03-11</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Piste identifiée</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2025-03-17</t>
+          <t>17/03/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>10/03/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2025-02-04</t>
+          <t>04/02/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>05/03/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2025-03-03</t>
+          <t>03/03/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2025-02-10</t>
+          <t>10/02/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Piste identifiée</t>
+          <t>Fermée</t>
         </is>
       </c>
     </row>

</xml_diff>